<commit_message>
Añadiendo importador de riesgo compañía
</commit_message>
<xml_diff>
--- a/krm/static/files/import_template.xlsx
+++ b/krm/static/files/import_template.xlsx
@@ -8,16 +8,17 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bienvenidosaez/Bitbucket/krm-kpmg/krm/static/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{64F066AB-C26E-E644-BFE0-324967697DF6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E3CB8DE7-43C6-814C-8F7B-98CF0143AFF3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="68260" yWindow="500" windowWidth="34140" windowHeight="27080" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="6640" yWindow="500" windowWidth="34140" windowHeight="27080" tabRatio="500" activeTab="4" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Domain Risk" sheetId="1" r:id="rId1"/>
-    <sheet name="Risk Master" sheetId="2" r:id="rId2"/>
-    <sheet name="Risk" sheetId="3" r:id="rId3"/>
+    <sheet name="Risk Master N1" sheetId="2" r:id="rId2"/>
+    <sheet name="Risk N2" sheetId="3" r:id="rId3"/>
     <sheet name="Controls" sheetId="5" r:id="rId4"/>
-    <sheet name="Avalibre values" sheetId="4" r:id="rId5"/>
+    <sheet name="RiskCompany" sheetId="6" r:id="rId5"/>
+    <sheet name="Avalibre values" sheetId="4" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -41,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="76" uniqueCount="69">
   <si>
     <t>L</t>
   </si>
@@ -300,6 +301,12 @@
   <si>
     <t>DOMAIN RISK REF</t>
   </si>
+  <si>
+    <t>Company REF</t>
+  </si>
+  <si>
+    <t>RISK N2 REF</t>
+  </si>
 </sst>
 </file>
 
@@ -385,7 +392,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="23">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
@@ -445,8 +452,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
@@ -761,7 +767,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="17.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="10" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.6640625" style="22"/>
+    <col min="2" max="2" width="17.6640625" style="3"/>
     <col min="3" max="3" width="50.83203125" style="2" customWidth="1"/>
     <col min="4" max="4" width="82.83203125" style="2" customWidth="1"/>
   </cols>
@@ -857,7 +863,7 @@
   <dimension ref="A1:L376"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="15.83203125" style="23" customWidth="1"/>
+    <col min="1" max="1" width="15.83203125" style="22" customWidth="1"/>
     <col min="2" max="2" width="21" style="18" customWidth="1"/>
     <col min="3" max="3" width="67.83203125" style="7" customWidth="1"/>
     <col min="4" max="4" width="72" style="1" customWidth="1"/>
@@ -5702,6 +5708,1528 @@
 </file>
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{78F0122E-3A36-E341-A4CC-5B5C3A26C773}">
+  <dimension ref="A1:B376"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="2" width="35" style="22" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A1" s="12" t="s">
+        <v>68</v>
+      </c>
+      <c r="B1" s="12" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A2" s="20"/>
+      <c r="B2" s="20"/>
+    </row>
+    <row r="3" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A3" s="20"/>
+      <c r="B3" s="20"/>
+    </row>
+    <row r="4" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A4" s="20"/>
+      <c r="B4" s="20"/>
+    </row>
+    <row r="5" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A5" s="20"/>
+      <c r="B5" s="20"/>
+    </row>
+    <row r="6" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A6" s="20"/>
+      <c r="B6" s="20"/>
+    </row>
+    <row r="7" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A7" s="20"/>
+      <c r="B7" s="20"/>
+    </row>
+    <row r="8" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A8" s="20"/>
+      <c r="B8" s="20"/>
+    </row>
+    <row r="9" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A9" s="20"/>
+      <c r="B9" s="20"/>
+    </row>
+    <row r="10" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A10" s="20"/>
+      <c r="B10" s="20"/>
+    </row>
+    <row r="11" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+    </row>
+    <row r="12" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A12" s="20"/>
+      <c r="B12" s="20"/>
+    </row>
+    <row r="13" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+    </row>
+    <row r="14" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A14" s="20"/>
+      <c r="B14" s="20"/>
+    </row>
+    <row r="15" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A15" s="20"/>
+      <c r="B15" s="20"/>
+    </row>
+    <row r="16" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A16" s="20"/>
+      <c r="B16" s="20"/>
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A17" s="20"/>
+      <c r="B17" s="20"/>
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A18" s="20"/>
+      <c r="B18" s="20"/>
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A19" s="20"/>
+      <c r="B19" s="20"/>
+    </row>
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A20" s="20"/>
+      <c r="B20" s="20"/>
+    </row>
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A21" s="20"/>
+      <c r="B21" s="20"/>
+    </row>
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A22" s="20"/>
+      <c r="B22" s="20"/>
+    </row>
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+    </row>
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A24" s="20"/>
+      <c r="B24" s="20"/>
+    </row>
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+    </row>
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A26" s="20"/>
+      <c r="B26" s="20"/>
+    </row>
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A27" s="20"/>
+      <c r="B27" s="20"/>
+    </row>
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A28" s="20"/>
+      <c r="B28" s="20"/>
+    </row>
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A29" s="20"/>
+      <c r="B29" s="20"/>
+    </row>
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A30" s="20"/>
+      <c r="B30" s="20"/>
+    </row>
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A31" s="20"/>
+      <c r="B31" s="20"/>
+    </row>
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A32" s="20"/>
+      <c r="B32" s="20"/>
+    </row>
+    <row r="33" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A33" s="20"/>
+      <c r="B33" s="20"/>
+    </row>
+    <row r="34" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A34" s="20"/>
+      <c r="B34" s="20"/>
+    </row>
+    <row r="35" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A35" s="20"/>
+      <c r="B35" s="20"/>
+    </row>
+    <row r="36" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A36" s="20"/>
+      <c r="B36" s="20"/>
+    </row>
+    <row r="37" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A37" s="20"/>
+      <c r="B37" s="20"/>
+    </row>
+    <row r="38" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A38" s="20"/>
+      <c r="B38" s="20"/>
+    </row>
+    <row r="39" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A39" s="20"/>
+      <c r="B39" s="20"/>
+    </row>
+    <row r="40" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A40" s="20"/>
+      <c r="B40" s="20"/>
+    </row>
+    <row r="41" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A41" s="20"/>
+      <c r="B41" s="20"/>
+    </row>
+    <row r="42" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A42" s="20"/>
+      <c r="B42" s="20"/>
+    </row>
+    <row r="43" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A43" s="20"/>
+      <c r="B43" s="20"/>
+    </row>
+    <row r="44" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A44" s="20"/>
+      <c r="B44" s="20"/>
+    </row>
+    <row r="45" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A45" s="20"/>
+      <c r="B45" s="20"/>
+    </row>
+    <row r="46" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A46" s="20"/>
+      <c r="B46" s="20"/>
+    </row>
+    <row r="47" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A47" s="20"/>
+      <c r="B47" s="20"/>
+    </row>
+    <row r="48" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A48" s="20"/>
+      <c r="B48" s="20"/>
+    </row>
+    <row r="49" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A49" s="20"/>
+      <c r="B49" s="20"/>
+    </row>
+    <row r="50" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A50" s="20"/>
+      <c r="B50" s="20"/>
+    </row>
+    <row r="51" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A51" s="20"/>
+      <c r="B51" s="20"/>
+    </row>
+    <row r="52" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A52" s="20"/>
+      <c r="B52" s="20"/>
+    </row>
+    <row r="53" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A53" s="20"/>
+      <c r="B53" s="20"/>
+    </row>
+    <row r="54" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A54" s="20"/>
+      <c r="B54" s="20"/>
+    </row>
+    <row r="55" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A55" s="20"/>
+      <c r="B55" s="20"/>
+    </row>
+    <row r="56" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A56" s="20"/>
+      <c r="B56" s="20"/>
+    </row>
+    <row r="57" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A57" s="20"/>
+      <c r="B57" s="20"/>
+    </row>
+    <row r="58" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A58" s="20"/>
+      <c r="B58" s="20"/>
+    </row>
+    <row r="59" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A59" s="20"/>
+      <c r="B59" s="20"/>
+    </row>
+    <row r="60" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A60" s="20"/>
+      <c r="B60" s="20"/>
+    </row>
+    <row r="61" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A61" s="20"/>
+      <c r="B61" s="20"/>
+    </row>
+    <row r="62" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A62" s="20"/>
+      <c r="B62" s="20"/>
+    </row>
+    <row r="63" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A63" s="20"/>
+      <c r="B63" s="20"/>
+    </row>
+    <row r="64" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A64" s="20"/>
+      <c r="B64" s="20"/>
+    </row>
+    <row r="65" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A65" s="20"/>
+      <c r="B65" s="20"/>
+    </row>
+    <row r="66" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A66" s="20"/>
+      <c r="B66" s="20"/>
+    </row>
+    <row r="67" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A67" s="20"/>
+      <c r="B67" s="20"/>
+    </row>
+    <row r="68" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A68" s="20"/>
+      <c r="B68" s="20"/>
+    </row>
+    <row r="69" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A69" s="20"/>
+      <c r="B69" s="20"/>
+    </row>
+    <row r="70" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A70" s="20"/>
+      <c r="B70" s="20"/>
+    </row>
+    <row r="71" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A71" s="20"/>
+      <c r="B71" s="20"/>
+    </row>
+    <row r="72" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A72" s="20"/>
+      <c r="B72" s="20"/>
+    </row>
+    <row r="73" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A73" s="20"/>
+      <c r="B73" s="20"/>
+    </row>
+    <row r="74" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A74" s="20"/>
+      <c r="B74" s="20"/>
+    </row>
+    <row r="75" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A75" s="20"/>
+      <c r="B75" s="20"/>
+    </row>
+    <row r="76" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A76" s="20"/>
+      <c r="B76" s="20"/>
+    </row>
+    <row r="77" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A77" s="20"/>
+      <c r="B77" s="20"/>
+    </row>
+    <row r="78" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A78" s="20"/>
+      <c r="B78" s="20"/>
+    </row>
+    <row r="79" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A79" s="20"/>
+      <c r="B79" s="20"/>
+    </row>
+    <row r="80" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A80" s="20"/>
+      <c r="B80" s="20"/>
+    </row>
+    <row r="81" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A81" s="20"/>
+      <c r="B81" s="20"/>
+    </row>
+    <row r="82" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A82" s="20"/>
+      <c r="B82" s="20"/>
+    </row>
+    <row r="83" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A83" s="20"/>
+      <c r="B83" s="20"/>
+    </row>
+    <row r="84" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A84" s="20"/>
+      <c r="B84" s="20"/>
+    </row>
+    <row r="85" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A85" s="20"/>
+      <c r="B85" s="20"/>
+    </row>
+    <row r="86" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A86" s="20"/>
+      <c r="B86" s="20"/>
+    </row>
+    <row r="87" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A87" s="20"/>
+      <c r="B87" s="20"/>
+    </row>
+    <row r="88" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A88" s="20"/>
+      <c r="B88" s="20"/>
+    </row>
+    <row r="89" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A89" s="20"/>
+      <c r="B89" s="20"/>
+    </row>
+    <row r="90" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A90" s="20"/>
+      <c r="B90" s="20"/>
+    </row>
+    <row r="91" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A91" s="20"/>
+      <c r="B91" s="20"/>
+    </row>
+    <row r="92" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A92" s="20"/>
+      <c r="B92" s="20"/>
+    </row>
+    <row r="93" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A93" s="20"/>
+      <c r="B93" s="20"/>
+    </row>
+    <row r="94" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A94" s="20"/>
+      <c r="B94" s="20"/>
+    </row>
+    <row r="95" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A95" s="20"/>
+      <c r="B95" s="20"/>
+    </row>
+    <row r="96" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A96" s="20"/>
+      <c r="B96" s="20"/>
+    </row>
+    <row r="97" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A97" s="20"/>
+      <c r="B97" s="20"/>
+    </row>
+    <row r="98" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A98" s="20"/>
+      <c r="B98" s="20"/>
+    </row>
+    <row r="99" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A99" s="20"/>
+      <c r="B99" s="20"/>
+    </row>
+    <row r="100" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A100" s="20"/>
+      <c r="B100" s="20"/>
+    </row>
+    <row r="101" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A101" s="20"/>
+      <c r="B101" s="20"/>
+    </row>
+    <row r="102" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A102" s="20"/>
+      <c r="B102" s="20"/>
+    </row>
+    <row r="103" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A103" s="20"/>
+      <c r="B103" s="20"/>
+    </row>
+    <row r="104" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A104" s="20"/>
+      <c r="B104" s="20"/>
+    </row>
+    <row r="105" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A105" s="20"/>
+      <c r="B105" s="20"/>
+    </row>
+    <row r="106" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A106" s="20"/>
+      <c r="B106" s="20"/>
+    </row>
+    <row r="107" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A107" s="20"/>
+      <c r="B107" s="20"/>
+    </row>
+    <row r="108" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A108" s="20"/>
+      <c r="B108" s="20"/>
+    </row>
+    <row r="109" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A109" s="20"/>
+      <c r="B109" s="20"/>
+    </row>
+    <row r="110" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A110" s="20"/>
+      <c r="B110" s="20"/>
+    </row>
+    <row r="111" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A111" s="20"/>
+      <c r="B111" s="20"/>
+    </row>
+    <row r="112" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A112" s="20"/>
+      <c r="B112" s="20"/>
+    </row>
+    <row r="113" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A113" s="20"/>
+      <c r="B113" s="20"/>
+    </row>
+    <row r="114" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A114" s="20"/>
+      <c r="B114" s="20"/>
+    </row>
+    <row r="115" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A115" s="20"/>
+      <c r="B115" s="20"/>
+    </row>
+    <row r="116" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A116" s="20"/>
+      <c r="B116" s="20"/>
+    </row>
+    <row r="117" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A117" s="20"/>
+      <c r="B117" s="20"/>
+    </row>
+    <row r="118" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A118" s="20"/>
+      <c r="B118" s="20"/>
+    </row>
+    <row r="119" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A119" s="20"/>
+      <c r="B119" s="20"/>
+    </row>
+    <row r="120" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A120" s="20"/>
+      <c r="B120" s="20"/>
+    </row>
+    <row r="121" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A121" s="20"/>
+      <c r="B121" s="20"/>
+    </row>
+    <row r="122" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A122" s="20"/>
+      <c r="B122" s="20"/>
+    </row>
+    <row r="123" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A123" s="20"/>
+      <c r="B123" s="20"/>
+    </row>
+    <row r="124" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A124" s="20"/>
+      <c r="B124" s="20"/>
+    </row>
+    <row r="125" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A125" s="20"/>
+      <c r="B125" s="20"/>
+    </row>
+    <row r="126" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A126" s="20"/>
+      <c r="B126" s="20"/>
+    </row>
+    <row r="127" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A127" s="20"/>
+      <c r="B127" s="20"/>
+    </row>
+    <row r="128" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A128" s="20"/>
+      <c r="B128" s="20"/>
+    </row>
+    <row r="129" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A129" s="20"/>
+      <c r="B129" s="20"/>
+    </row>
+    <row r="130" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A130" s="20"/>
+      <c r="B130" s="20"/>
+    </row>
+    <row r="131" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A131" s="20"/>
+      <c r="B131" s="20"/>
+    </row>
+    <row r="132" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A132" s="20"/>
+      <c r="B132" s="20"/>
+    </row>
+    <row r="133" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A133" s="20"/>
+      <c r="B133" s="20"/>
+    </row>
+    <row r="134" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A134" s="20"/>
+      <c r="B134" s="20"/>
+    </row>
+    <row r="135" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A135" s="20"/>
+      <c r="B135" s="20"/>
+    </row>
+    <row r="136" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A136" s="20"/>
+      <c r="B136" s="20"/>
+    </row>
+    <row r="137" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A137" s="20"/>
+      <c r="B137" s="20"/>
+    </row>
+    <row r="138" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A138" s="20"/>
+      <c r="B138" s="20"/>
+    </row>
+    <row r="139" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A139" s="20"/>
+      <c r="B139" s="20"/>
+    </row>
+    <row r="140" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A140" s="20"/>
+      <c r="B140" s="20"/>
+    </row>
+    <row r="141" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A141" s="20"/>
+      <c r="B141" s="20"/>
+    </row>
+    <row r="142" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A142" s="20"/>
+      <c r="B142" s="20"/>
+    </row>
+    <row r="143" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A143" s="20"/>
+      <c r="B143" s="20"/>
+    </row>
+    <row r="144" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A144" s="20"/>
+      <c r="B144" s="20"/>
+    </row>
+    <row r="145" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A145" s="20"/>
+      <c r="B145" s="20"/>
+    </row>
+    <row r="146" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A146" s="20"/>
+      <c r="B146" s="20"/>
+    </row>
+    <row r="147" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A147" s="20"/>
+      <c r="B147" s="20"/>
+    </row>
+    <row r="148" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A148" s="20"/>
+      <c r="B148" s="20"/>
+    </row>
+    <row r="149" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A149" s="20"/>
+      <c r="B149" s="20"/>
+    </row>
+    <row r="150" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A150" s="20"/>
+      <c r="B150" s="20"/>
+    </row>
+    <row r="151" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A151" s="20"/>
+      <c r="B151" s="20"/>
+    </row>
+    <row r="152" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A152" s="20"/>
+      <c r="B152" s="20"/>
+    </row>
+    <row r="153" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A153" s="20"/>
+      <c r="B153" s="20"/>
+    </row>
+    <row r="154" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A154" s="20"/>
+      <c r="B154" s="20"/>
+    </row>
+    <row r="155" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A155" s="20"/>
+      <c r="B155" s="20"/>
+    </row>
+    <row r="156" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A156" s="20"/>
+      <c r="B156" s="20"/>
+    </row>
+    <row r="157" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A157" s="20"/>
+      <c r="B157" s="20"/>
+    </row>
+    <row r="158" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A158" s="20"/>
+      <c r="B158" s="20"/>
+    </row>
+    <row r="159" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A159" s="20"/>
+      <c r="B159" s="20"/>
+    </row>
+    <row r="160" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A160" s="20"/>
+      <c r="B160" s="20"/>
+    </row>
+    <row r="161" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A161" s="20"/>
+      <c r="B161" s="20"/>
+    </row>
+    <row r="162" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A162" s="20"/>
+      <c r="B162" s="20"/>
+    </row>
+    <row r="163" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A163" s="20"/>
+      <c r="B163" s="20"/>
+    </row>
+    <row r="164" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A164" s="20"/>
+      <c r="B164" s="20"/>
+    </row>
+    <row r="165" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A165" s="20"/>
+      <c r="B165" s="20"/>
+    </row>
+    <row r="166" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A166" s="20"/>
+      <c r="B166" s="20"/>
+    </row>
+    <row r="167" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A167" s="20"/>
+      <c r="B167" s="20"/>
+    </row>
+    <row r="168" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A168" s="20"/>
+      <c r="B168" s="20"/>
+    </row>
+    <row r="169" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A169" s="20"/>
+      <c r="B169" s="20"/>
+    </row>
+    <row r="170" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A170" s="20"/>
+      <c r="B170" s="20"/>
+    </row>
+    <row r="171" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A171" s="20"/>
+      <c r="B171" s="20"/>
+    </row>
+    <row r="172" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A172" s="20"/>
+      <c r="B172" s="20"/>
+    </row>
+    <row r="173" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A173" s="20"/>
+      <c r="B173" s="20"/>
+    </row>
+    <row r="174" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A174" s="20"/>
+      <c r="B174" s="20"/>
+    </row>
+    <row r="175" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A175" s="20"/>
+      <c r="B175" s="20"/>
+    </row>
+    <row r="176" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A176" s="20"/>
+      <c r="B176" s="20"/>
+    </row>
+    <row r="177" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A177" s="20"/>
+      <c r="B177" s="20"/>
+    </row>
+    <row r="178" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A178" s="20"/>
+      <c r="B178" s="20"/>
+    </row>
+    <row r="179" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A179" s="20"/>
+      <c r="B179" s="20"/>
+    </row>
+    <row r="180" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A180" s="20"/>
+      <c r="B180" s="20"/>
+    </row>
+    <row r="181" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A181" s="20"/>
+      <c r="B181" s="20"/>
+    </row>
+    <row r="182" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A182" s="20"/>
+      <c r="B182" s="20"/>
+    </row>
+    <row r="183" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A183" s="20"/>
+      <c r="B183" s="20"/>
+    </row>
+    <row r="184" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A184" s="20"/>
+      <c r="B184" s="20"/>
+    </row>
+    <row r="185" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A185" s="20"/>
+      <c r="B185" s="20"/>
+    </row>
+    <row r="186" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A186" s="20"/>
+      <c r="B186" s="20"/>
+    </row>
+    <row r="187" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A187" s="20"/>
+      <c r="B187" s="20"/>
+    </row>
+    <row r="188" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A188" s="20"/>
+      <c r="B188" s="20"/>
+    </row>
+    <row r="189" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A189" s="20"/>
+      <c r="B189" s="20"/>
+    </row>
+    <row r="190" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A190" s="20"/>
+      <c r="B190" s="20"/>
+    </row>
+    <row r="191" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A191" s="20"/>
+      <c r="B191" s="20"/>
+    </row>
+    <row r="192" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A192" s="20"/>
+      <c r="B192" s="20"/>
+    </row>
+    <row r="193" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A193" s="20"/>
+      <c r="B193" s="20"/>
+    </row>
+    <row r="194" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A194" s="20"/>
+      <c r="B194" s="20"/>
+    </row>
+    <row r="195" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A195" s="20"/>
+      <c r="B195" s="20"/>
+    </row>
+    <row r="196" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A196" s="20"/>
+      <c r="B196" s="20"/>
+    </row>
+    <row r="197" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A197" s="20"/>
+      <c r="B197" s="20"/>
+    </row>
+    <row r="198" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A198" s="20"/>
+      <c r="B198" s="20"/>
+    </row>
+    <row r="199" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A199" s="20"/>
+      <c r="B199" s="20"/>
+    </row>
+    <row r="200" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A200" s="20"/>
+      <c r="B200" s="20"/>
+    </row>
+    <row r="201" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A201" s="20"/>
+      <c r="B201" s="20"/>
+    </row>
+    <row r="202" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A202" s="20"/>
+      <c r="B202" s="20"/>
+    </row>
+    <row r="203" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A203" s="20"/>
+      <c r="B203" s="20"/>
+    </row>
+    <row r="204" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A204" s="20"/>
+      <c r="B204" s="20"/>
+    </row>
+    <row r="205" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A205" s="20"/>
+      <c r="B205" s="20"/>
+    </row>
+    <row r="206" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A206" s="20"/>
+      <c r="B206" s="20"/>
+    </row>
+    <row r="207" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A207" s="20"/>
+      <c r="B207" s="20"/>
+    </row>
+    <row r="208" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A208" s="20"/>
+      <c r="B208" s="20"/>
+    </row>
+    <row r="209" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A209" s="20"/>
+      <c r="B209" s="20"/>
+    </row>
+    <row r="210" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A210" s="20"/>
+      <c r="B210" s="20"/>
+    </row>
+    <row r="211" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A211" s="20"/>
+      <c r="B211" s="20"/>
+    </row>
+    <row r="212" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A212" s="20"/>
+      <c r="B212" s="20"/>
+    </row>
+    <row r="213" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A213" s="20"/>
+      <c r="B213" s="20"/>
+    </row>
+    <row r="214" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A214" s="20"/>
+      <c r="B214" s="20"/>
+    </row>
+    <row r="215" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A215" s="20"/>
+      <c r="B215" s="20"/>
+    </row>
+    <row r="216" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A216" s="20"/>
+      <c r="B216" s="20"/>
+    </row>
+    <row r="217" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A217" s="20"/>
+      <c r="B217" s="20"/>
+    </row>
+    <row r="218" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A218" s="20"/>
+      <c r="B218" s="20"/>
+    </row>
+    <row r="219" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A219" s="20"/>
+      <c r="B219" s="20"/>
+    </row>
+    <row r="220" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A220" s="20"/>
+      <c r="B220" s="20"/>
+    </row>
+    <row r="221" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A221" s="20"/>
+      <c r="B221" s="20"/>
+    </row>
+    <row r="222" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A222" s="20"/>
+      <c r="B222" s="20"/>
+    </row>
+    <row r="223" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A223" s="20"/>
+      <c r="B223" s="20"/>
+    </row>
+    <row r="224" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A224" s="20"/>
+      <c r="B224" s="20"/>
+    </row>
+    <row r="225" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A225" s="20"/>
+      <c r="B225" s="20"/>
+    </row>
+    <row r="226" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A226" s="20"/>
+      <c r="B226" s="20"/>
+    </row>
+    <row r="227" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A227" s="20"/>
+      <c r="B227" s="20"/>
+    </row>
+    <row r="228" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A228" s="20"/>
+      <c r="B228" s="20"/>
+    </row>
+    <row r="229" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A229" s="20"/>
+      <c r="B229" s="20"/>
+    </row>
+    <row r="230" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A230" s="20"/>
+      <c r="B230" s="20"/>
+    </row>
+    <row r="231" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A231" s="20"/>
+      <c r="B231" s="20"/>
+    </row>
+    <row r="232" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A232" s="20"/>
+      <c r="B232" s="20"/>
+    </row>
+    <row r="233" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A233" s="20"/>
+      <c r="B233" s="20"/>
+    </row>
+    <row r="234" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A234" s="20"/>
+      <c r="B234" s="20"/>
+    </row>
+    <row r="235" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A235" s="20"/>
+      <c r="B235" s="20"/>
+    </row>
+    <row r="236" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A236" s="20"/>
+      <c r="B236" s="20"/>
+    </row>
+    <row r="237" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A237" s="20"/>
+      <c r="B237" s="20"/>
+    </row>
+    <row r="238" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A238" s="20"/>
+      <c r="B238" s="20"/>
+    </row>
+    <row r="239" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A239" s="20"/>
+      <c r="B239" s="20"/>
+    </row>
+    <row r="240" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A240" s="20"/>
+      <c r="B240" s="20"/>
+    </row>
+    <row r="241" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A241" s="20"/>
+      <c r="B241" s="20"/>
+    </row>
+    <row r="242" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A242" s="20"/>
+      <c r="B242" s="20"/>
+    </row>
+    <row r="243" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A243" s="20"/>
+      <c r="B243" s="20"/>
+    </row>
+    <row r="244" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A244" s="20"/>
+      <c r="B244" s="20"/>
+    </row>
+    <row r="245" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A245" s="20"/>
+      <c r="B245" s="20"/>
+    </row>
+    <row r="246" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A246" s="20"/>
+      <c r="B246" s="20"/>
+    </row>
+    <row r="247" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A247" s="20"/>
+      <c r="B247" s="20"/>
+    </row>
+    <row r="248" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A248" s="20"/>
+      <c r="B248" s="20"/>
+    </row>
+    <row r="249" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A249" s="20"/>
+      <c r="B249" s="20"/>
+    </row>
+    <row r="250" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A250" s="20"/>
+      <c r="B250" s="20"/>
+    </row>
+    <row r="251" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A251" s="20"/>
+      <c r="B251" s="20"/>
+    </row>
+    <row r="252" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A252" s="20"/>
+      <c r="B252" s="20"/>
+    </row>
+    <row r="253" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A253" s="20"/>
+      <c r="B253" s="20"/>
+    </row>
+    <row r="254" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A254" s="20"/>
+      <c r="B254" s="20"/>
+    </row>
+    <row r="255" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A255" s="20"/>
+      <c r="B255" s="20"/>
+    </row>
+    <row r="256" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A256" s="20"/>
+      <c r="B256" s="20"/>
+    </row>
+    <row r="257" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A257" s="20"/>
+      <c r="B257" s="20"/>
+    </row>
+    <row r="258" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A258" s="20"/>
+      <c r="B258" s="20"/>
+    </row>
+    <row r="259" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A259" s="20"/>
+      <c r="B259" s="20"/>
+    </row>
+    <row r="260" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A260" s="20"/>
+      <c r="B260" s="20"/>
+    </row>
+    <row r="261" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A261" s="20"/>
+      <c r="B261" s="20"/>
+    </row>
+    <row r="262" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A262" s="20"/>
+      <c r="B262" s="20"/>
+    </row>
+    <row r="263" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A263" s="20"/>
+      <c r="B263" s="20"/>
+    </row>
+    <row r="264" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A264" s="20"/>
+      <c r="B264" s="20"/>
+    </row>
+    <row r="265" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A265" s="20"/>
+      <c r="B265" s="20"/>
+    </row>
+    <row r="266" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A266" s="20"/>
+      <c r="B266" s="20"/>
+    </row>
+    <row r="267" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A267" s="20"/>
+      <c r="B267" s="20"/>
+    </row>
+    <row r="268" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A268" s="20"/>
+      <c r="B268" s="20"/>
+    </row>
+    <row r="269" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A269" s="20"/>
+      <c r="B269" s="20"/>
+    </row>
+    <row r="270" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A270" s="20"/>
+      <c r="B270" s="20"/>
+    </row>
+    <row r="271" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A271" s="20"/>
+      <c r="B271" s="20"/>
+    </row>
+    <row r="272" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A272" s="20"/>
+      <c r="B272" s="20"/>
+    </row>
+    <row r="273" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A273" s="20"/>
+      <c r="B273" s="20"/>
+    </row>
+    <row r="274" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A274" s="20"/>
+      <c r="B274" s="20"/>
+    </row>
+    <row r="275" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A275" s="20"/>
+      <c r="B275" s="20"/>
+    </row>
+    <row r="276" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A276" s="20"/>
+      <c r="B276" s="20"/>
+    </row>
+    <row r="277" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A277" s="20"/>
+      <c r="B277" s="20"/>
+    </row>
+    <row r="278" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A278" s="20"/>
+      <c r="B278" s="20"/>
+    </row>
+    <row r="279" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A279" s="20"/>
+      <c r="B279" s="20"/>
+    </row>
+    <row r="280" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A280" s="20"/>
+      <c r="B280" s="20"/>
+    </row>
+    <row r="281" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A281" s="20"/>
+      <c r="B281" s="20"/>
+    </row>
+    <row r="282" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A282" s="20"/>
+      <c r="B282" s="20"/>
+    </row>
+    <row r="283" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A283" s="20"/>
+      <c r="B283" s="20"/>
+    </row>
+    <row r="284" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A284" s="20"/>
+      <c r="B284" s="20"/>
+    </row>
+    <row r="285" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A285" s="20"/>
+      <c r="B285" s="20"/>
+    </row>
+    <row r="286" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A286" s="20"/>
+      <c r="B286" s="20"/>
+    </row>
+    <row r="287" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A287" s="20"/>
+      <c r="B287" s="20"/>
+    </row>
+    <row r="288" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A288" s="20"/>
+      <c r="B288" s="20"/>
+    </row>
+    <row r="289" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A289" s="20"/>
+      <c r="B289" s="20"/>
+    </row>
+    <row r="290" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A290" s="20"/>
+      <c r="B290" s="20"/>
+    </row>
+    <row r="291" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A291" s="20"/>
+      <c r="B291" s="20"/>
+    </row>
+    <row r="292" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A292" s="20"/>
+      <c r="B292" s="20"/>
+    </row>
+    <row r="293" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A293" s="20"/>
+      <c r="B293" s="20"/>
+    </row>
+    <row r="294" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A294" s="20"/>
+      <c r="B294" s="20"/>
+    </row>
+    <row r="295" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A295" s="20"/>
+      <c r="B295" s="20"/>
+    </row>
+    <row r="296" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A296" s="20"/>
+      <c r="B296" s="20"/>
+    </row>
+    <row r="297" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A297" s="20"/>
+      <c r="B297" s="20"/>
+    </row>
+    <row r="298" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A298" s="20"/>
+      <c r="B298" s="20"/>
+    </row>
+    <row r="299" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A299" s="20"/>
+      <c r="B299" s="20"/>
+    </row>
+    <row r="300" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A300" s="20"/>
+      <c r="B300" s="20"/>
+    </row>
+    <row r="301" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A301" s="20"/>
+      <c r="B301" s="20"/>
+    </row>
+    <row r="302" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A302" s="20"/>
+      <c r="B302" s="20"/>
+    </row>
+    <row r="303" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A303" s="20"/>
+      <c r="B303" s="20"/>
+    </row>
+    <row r="304" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A304" s="20"/>
+      <c r="B304" s="20"/>
+    </row>
+    <row r="305" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A305" s="20"/>
+      <c r="B305" s="20"/>
+    </row>
+    <row r="306" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A306" s="20"/>
+      <c r="B306" s="20"/>
+    </row>
+    <row r="307" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A307" s="20"/>
+      <c r="B307" s="20"/>
+    </row>
+    <row r="308" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A308" s="20"/>
+      <c r="B308" s="20"/>
+    </row>
+    <row r="309" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A309" s="20"/>
+      <c r="B309" s="20"/>
+    </row>
+    <row r="310" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A310" s="20"/>
+      <c r="B310" s="20"/>
+    </row>
+    <row r="311" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A311" s="20"/>
+      <c r="B311" s="20"/>
+    </row>
+    <row r="312" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A312" s="20"/>
+      <c r="B312" s="20"/>
+    </row>
+    <row r="313" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A313" s="20"/>
+      <c r="B313" s="20"/>
+    </row>
+    <row r="314" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A314" s="20"/>
+      <c r="B314" s="20"/>
+    </row>
+    <row r="315" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A315" s="20"/>
+      <c r="B315" s="20"/>
+    </row>
+    <row r="316" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A316" s="20"/>
+      <c r="B316" s="20"/>
+    </row>
+    <row r="317" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A317" s="20"/>
+      <c r="B317" s="20"/>
+    </row>
+    <row r="318" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A318" s="20"/>
+      <c r="B318" s="20"/>
+    </row>
+    <row r="319" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A319" s="20"/>
+      <c r="B319" s="20"/>
+    </row>
+    <row r="320" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A320" s="20"/>
+      <c r="B320" s="20"/>
+    </row>
+    <row r="321" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A321" s="20"/>
+      <c r="B321" s="20"/>
+    </row>
+    <row r="322" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A322" s="20"/>
+      <c r="B322" s="20"/>
+    </row>
+    <row r="323" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A323" s="20"/>
+      <c r="B323" s="20"/>
+    </row>
+    <row r="324" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A324" s="20"/>
+      <c r="B324" s="20"/>
+    </row>
+    <row r="325" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A325" s="20"/>
+      <c r="B325" s="20"/>
+    </row>
+    <row r="326" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A326" s="20"/>
+      <c r="B326" s="20"/>
+    </row>
+    <row r="327" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A327" s="20"/>
+      <c r="B327" s="20"/>
+    </row>
+    <row r="328" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A328" s="20"/>
+      <c r="B328" s="20"/>
+    </row>
+    <row r="329" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A329" s="20"/>
+      <c r="B329" s="20"/>
+    </row>
+    <row r="330" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A330" s="20"/>
+      <c r="B330" s="20"/>
+    </row>
+    <row r="331" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A331" s="20"/>
+      <c r="B331" s="20"/>
+    </row>
+    <row r="332" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A332" s="20"/>
+      <c r="B332" s="20"/>
+    </row>
+    <row r="333" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A333" s="20"/>
+      <c r="B333" s="20"/>
+    </row>
+    <row r="334" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A334" s="20"/>
+      <c r="B334" s="20"/>
+    </row>
+    <row r="335" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A335" s="20"/>
+      <c r="B335" s="20"/>
+    </row>
+    <row r="336" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A336" s="20"/>
+      <c r="B336" s="20"/>
+    </row>
+    <row r="337" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A337" s="20"/>
+      <c r="B337" s="20"/>
+    </row>
+    <row r="338" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A338" s="20"/>
+      <c r="B338" s="20"/>
+    </row>
+    <row r="339" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A339" s="20"/>
+      <c r="B339" s="20"/>
+    </row>
+    <row r="340" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A340" s="20"/>
+      <c r="B340" s="20"/>
+    </row>
+    <row r="341" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A341" s="20"/>
+      <c r="B341" s="20"/>
+    </row>
+    <row r="342" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A342" s="20"/>
+      <c r="B342" s="20"/>
+    </row>
+    <row r="343" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A343" s="20"/>
+      <c r="B343" s="20"/>
+    </row>
+    <row r="344" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A344" s="20"/>
+      <c r="B344" s="20"/>
+    </row>
+    <row r="345" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A345" s="20"/>
+      <c r="B345" s="20"/>
+    </row>
+    <row r="346" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A346" s="20"/>
+      <c r="B346" s="20"/>
+    </row>
+    <row r="347" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A347" s="20"/>
+      <c r="B347" s="20"/>
+    </row>
+    <row r="348" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A348" s="20"/>
+      <c r="B348" s="20"/>
+    </row>
+    <row r="349" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A349" s="20"/>
+      <c r="B349" s="20"/>
+    </row>
+    <row r="350" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A350" s="20"/>
+      <c r="B350" s="20"/>
+    </row>
+    <row r="351" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A351" s="20"/>
+      <c r="B351" s="20"/>
+    </row>
+    <row r="352" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A352" s="20"/>
+      <c r="B352" s="20"/>
+    </row>
+    <row r="353" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A353" s="20"/>
+      <c r="B353" s="20"/>
+    </row>
+    <row r="354" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A354" s="20"/>
+      <c r="B354" s="20"/>
+    </row>
+    <row r="355" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A355" s="20"/>
+      <c r="B355" s="20"/>
+    </row>
+    <row r="356" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A356" s="20"/>
+      <c r="B356" s="20"/>
+    </row>
+    <row r="357" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A357" s="20"/>
+      <c r="B357" s="20"/>
+    </row>
+    <row r="358" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A358" s="20"/>
+      <c r="B358" s="20"/>
+    </row>
+    <row r="359" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A359" s="20"/>
+      <c r="B359" s="20"/>
+    </row>
+    <row r="360" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A360" s="20"/>
+      <c r="B360" s="20"/>
+    </row>
+    <row r="361" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A361" s="20"/>
+      <c r="B361" s="20"/>
+    </row>
+    <row r="362" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A362" s="20"/>
+      <c r="B362" s="20"/>
+    </row>
+    <row r="363" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A363" s="20"/>
+      <c r="B363" s="20"/>
+    </row>
+    <row r="364" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A364" s="20"/>
+      <c r="B364" s="20"/>
+    </row>
+    <row r="365" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A365" s="20"/>
+      <c r="B365" s="20"/>
+    </row>
+    <row r="366" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A366" s="20"/>
+      <c r="B366" s="20"/>
+    </row>
+    <row r="367" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A367" s="20"/>
+      <c r="B367" s="20"/>
+    </row>
+    <row r="368" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A368" s="20"/>
+      <c r="B368" s="20"/>
+    </row>
+    <row r="369" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A369" s="20"/>
+      <c r="B369" s="20"/>
+    </row>
+    <row r="370" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A370" s="20"/>
+      <c r="B370" s="20"/>
+    </row>
+    <row r="371" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A371" s="20"/>
+      <c r="B371" s="20"/>
+    </row>
+    <row r="372" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A372" s="20"/>
+      <c r="B372" s="20"/>
+    </row>
+    <row r="373" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A373" s="20"/>
+      <c r="B373" s="20"/>
+    </row>
+    <row r="374" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A374" s="20"/>
+      <c r="B374" s="20"/>
+    </row>
+    <row r="375" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A375" s="20"/>
+      <c r="B375" s="20"/>
+    </row>
+    <row r="376" spans="1:2" x14ac:dyDescent="0.2">
+      <c r="A376" s="20"/>
+      <c r="B376" s="20"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" horizontalDpi="0" verticalDpi="0"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:I9"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>

</xml_diff>

<commit_message>
Attr ELC cambio plantilla importacion
</commit_message>
<xml_diff>
--- a/krm/static/files/import_template.xlsx
+++ b/krm/static/files/import_template.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/bienvenidosaez/Bitbucket/krm-kpmg/krm/static/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{9B8C9B9F-62E2-DA47-A233-AD1CE552912E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{22FD65A7-0DC2-A840-A9EB-1EEC35956AD0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2720" yWindow="6000" windowWidth="47840" windowHeight="24200" tabRatio="500" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2720" yWindow="3380" windowWidth="47840" windowHeight="24200" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Domain Risk" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="84" uniqueCount="70">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="71">
   <si>
     <t>L</t>
   </si>
@@ -310,6 +310,9 @@
   </si>
   <si>
     <t>CONTROL REF</t>
+  </si>
+  <si>
+    <t>ELC</t>
   </si>
 </sst>
 </file>
@@ -5577,7 +5580,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
-  <dimension ref="A1:S1"/>
+  <dimension ref="A1:T1"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.6640625" defaultRowHeight="16" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="35.6640625" style="10" customWidth="1"/>
@@ -5598,10 +5601,10 @@
     <col min="16" max="16" width="14" style="2" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="11.5" style="2" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="9.33203125" style="2" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="5.83203125" style="2" bestFit="1" customWidth="1"/>
+    <col min="19" max="20" width="5.83203125" style="2" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" s="6" customFormat="1" ht="153" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:20" s="6" customFormat="1" ht="153" x14ac:dyDescent="0.2">
       <c r="A1" s="17" t="s">
         <v>64</v>
       </c>
@@ -5659,6 +5662,9 @@
       <c r="S1" s="8" t="s">
         <v>9</v>
       </c>
+      <c r="T1" s="8" t="s">
+        <v>70</v>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="4">
@@ -5703,7 +5709,7 @@
           <x14:formula1>
             <xm:f>'Avalibre values'!$I$2:$I$4</xm:f>
           </x14:formula1>
-          <xm:sqref>L2:S200</xm:sqref>
+          <xm:sqref>L2:T200</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>

</xml_diff>

<commit_message>
Commit con los cambios a día 07/05
</commit_message>
<xml_diff>
--- a/krm/static/files/import_template.xlsx
+++ b/krm/static/files/import_template.xlsx
@@ -5,19 +5,19 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\nataliamonsalve\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://onedrive-global.kpmg.com/personal/nataliamonsalve_kpmg_es/Documents/Documents/Repositorios Git/dev-sidenor/krm/static/files/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{747F8EE9-8D6F-471A-8A7B-6F7541E77644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="1" documentId="13_ncr:1_{747F8EE9-8D6F-471A-8A7B-6F7541E77644}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{349CF1AC-F571-47BC-99CB-D3CAF5ABE302}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="3" activeTab="8" xr2:uid="{3BA6850B-93BC-4A7E-8C7E-92CACC72CE03}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10420" firstSheet="1" activeTab="6" xr2:uid="{3BA6850B-93BC-4A7E-8C7E-92CACC72CE03}"/>
   </bookViews>
   <sheets>
     <sheet name="Domain Risks" sheetId="2" r:id="rId1"/>
     <sheet name="Master Risks N1" sheetId="3" r:id="rId2"/>
     <sheet name="Risks N2" sheetId="4" r:id="rId3"/>
-    <sheet name="Company Risks" sheetId="7" r:id="rId4"/>
-    <sheet name="Processes" sheetId="9" r:id="rId5"/>
+    <sheet name="Processes" sheetId="9" r:id="rId4"/>
+    <sheet name="Company Risks" sheetId="7" r:id="rId5"/>
     <sheet name="Subprocesses" sheetId="10" r:id="rId6"/>
     <sheet name="Controls" sheetId="5" r:id="rId7"/>
     <sheet name="Company Controls" sheetId="6" r:id="rId8"/>
@@ -3896,6 +3896,49 @@
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E940B3B-6DF3-4CD7-89D4-35260A2B1441}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="8.7265625" style="8"/>
+    <col min="2" max="2" width="19.453125" style="8" customWidth="1"/>
+    <col min="3" max="3" width="21.26953125" style="8" customWidth="1"/>
+    <col min="4" max="16384" width="8.7265625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="3" t="s">
+        <v>92</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" s="15"/>
+      <c r="B2" s="15"/>
+      <c r="C2" s="15"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" s="15"/>
+      <c r="B3" s="15"/>
+      <c r="C3" s="15"/>
+      <c r="F3" s="11"/>
+    </row>
+  </sheetData>
+  <dataValidations count="3">
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Process Ref" prompt="The entered value must be an alphanumeric value up to 140 characters_x000a_" sqref="A1:A1048576" xr:uid="{16AEF36D-A31C-43D2-ACA8-120F6C1986C8}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Process Name" prompt="The entered value must be an alphanumeric value up to 500 characters_x000a_" sqref="B1:B1048576" xr:uid="{F840E8B1-390E-4F6F-A905-4446992BCF88}"/>
+    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Process Description" prompt="It must not exceed 10,000 characters in length_x000a_" sqref="C1:C1048576" xr:uid="{F3A710A8-E644-4E08-BA52-87E6E7D32425}"/>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2A215C40-C23E-48D8-A758-E0901DB62E1C}">
   <dimension ref="A1:J376"/>
   <sheetFormatPr defaultColWidth="11.453125" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
@@ -7831,49 +7874,6 @@
   </dataValidations>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" horizontalDpi="300" verticalDpi="300"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8E940B3B-6DF3-4CD7-89D4-35260A2B1441}">
-  <dimension ref="A1:F3"/>
-  <sheetFormatPr defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
-  <cols>
-    <col min="1" max="1" width="8.7265625" style="8"/>
-    <col min="2" max="2" width="19.453125" style="8" customWidth="1"/>
-    <col min="3" max="3" width="21.26953125" style="8" customWidth="1"/>
-    <col min="4" max="16384" width="8.7265625" style="1"/>
-  </cols>
-  <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A1" s="3" t="s">
-        <v>92</v>
-      </c>
-      <c r="B1" s="3" t="s">
-        <v>93</v>
-      </c>
-      <c r="C1" s="3" t="s">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A2" s="15"/>
-      <c r="B2" s="15"/>
-      <c r="C2" s="15"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A3" s="15"/>
-      <c r="B3" s="15"/>
-      <c r="C3" s="15"/>
-      <c r="F3" s="11"/>
-    </row>
-  </sheetData>
-  <dataValidations count="3">
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Process Ref" prompt="The entered value must be an alphanumeric value up to 140 characters_x000a_" sqref="A1:A1048576" xr:uid="{16AEF36D-A31C-43D2-ACA8-120F6C1986C8}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Process Name" prompt="The entered value must be an alphanumeric value up to 500 characters_x000a_" sqref="B1:B1048576" xr:uid="{F840E8B1-390E-4F6F-A905-4446992BCF88}"/>
-    <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" promptTitle="Process Description" prompt="It must not exceed 10,000 characters in length_x000a_" sqref="C1:C1048576" xr:uid="{F3A710A8-E644-4E08-BA52-87E6E7D32425}"/>
-  </dataValidations>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
@@ -10728,23 +10728,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <_activity xmlns="2281df0c-1fa8-44a4-821a-eaeb33136926" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
-</file>
-
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100AC7800D64BD77F40AEFD51E571CB5BF9" ma:contentTypeVersion="9" ma:contentTypeDescription="Create a new document." ma:contentTypeScope="" ma:versionID="47e31ca7aa67512d3cb50f66b2ca6b74">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns3="2281df0c-1fa8-44a4-821a-eaeb33136926" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="5d5ddb5a77c51ae7bb9ea3f55e4d744f" ns3:_="">
     <xsd:import namespace="2281df0c-1fa8-44a4-821a-eaeb33136926"/>
@@ -10920,10 +10903,37 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <_activity xmlns="2281df0c-1fa8-44a4-821a-eaeb33136926" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B32E056-F715-4218-89CD-3375EE5965A5}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24DBBF7B-BF59-458B-B194-B18D3D857E80}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="2281df0c-1fa8-44a4-821a-eaeb33136926"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -10945,19 +10955,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{24DBBF7B-BF59-458B-B194-B18D3D857E80}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{9B32E056-F715-4218-89CD-3375EE5965A5}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="2281df0c-1fa8-44a4-821a-eaeb33136926"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>